<commit_message>
Reconcile Resources public artifacts and workbook parity
Layer the independently verified Resources artifact candidate onto the concurrent review branch without discarding its additional templates, indexes or staging-preview links. Correct Family Emergency wording, publish the verified Export Check 1.2.0 workbook at a versioned path, retain rehearsal.xlsx as a byte-identical compatibility alias, and align portable JSON/CSV examples and human instructions. Preserve existing licence decisions and machine taxonomy files. Review branch only; no public-main or production promotion.
</commit_message>
<xml_diff>
--- a/checklists/family-emergency-document-checklist/checklist.xlsx
+++ b/checklists/family-emergency-document-checklist/checklist.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checklist'!$A$1:$G$30</definedName>
   </definedNames>
-  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,57 +88,8 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF1F2937"/>
-      <sz val="20"/>
-    </font>
-    <font>
-      <color rgb="FF6B7280"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="FF111827"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF0F766E"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <color rgb="FF111827"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF1F2937"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF9A3412"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF0F766E"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF111827"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF111827"/>
-    </font>
   </fonts>
-  <fills count="12">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -170,31 +121,6 @@
         <fgColor rgb="00F9FAFB"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE6F4F1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEDD5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF7ED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F2937"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF9FAFB"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -219,7 +145,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -268,48 +194,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -677,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A2:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -685,125 +577,119 @@
     <col width="90" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="30" customHeight="1">
       <c r="B2" s="20" t="inlineStr">
         <is>
           <t>Family Emergency Document Checklist</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="20" customHeight="1">
       <c r="B3" s="21" t="inlineStr">
         <is>
-          <t>Version 0.1.1 | Reviewed 17 September 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+          <t>Maintenance candidate 0.1.1</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="B5" s="22" t="inlineStr">
-        <is>
-          <t>Make the most important contacts and information easy to find when normal routines are disrupted. You do not need to carry every document.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>The point is not to carry every important document. The point is to make the few things that matter findable and usable when normal routines break.</t>
+        </is>
+      </c>
+    </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>1. Know where it is</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
-        <is>
-          <t>Someone you trust can find the current record when it is needed.</t>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Someone can locate the current or original record when it is needed.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>2. Keep the useful part accessible</t>
         </is>
       </c>
-      <c r="C8" s="24" t="inlineStr">
-        <is>
-          <t>Keep the contact details, short notes or useful copies needed in the first hours easy to reach.</t>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>The phone number, reference number, short summary or appropriate copy that helps in the first hours can be reached quickly.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>3. Protect the original</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>Keep sensitive originals in their usual secure place unless you need to move them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Sensitive originals stay in their normal secure home unless there is a real reason to move them.</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
-      <c r="B12" s="25" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>If you only have 15 minutes</t>
         </is>
       </c>
     </row>
     <row r="13" ht="72" customHeight="1">
-      <c r="B13" s="26" t="inlineStr">
-        <is>
-          <t>Start with contacts and meeting places, medication and care information, insurance details, important-document locations, dependant or pet arrangements, and your emergency-kit location.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="B15" s="27" t="inlineStr">
-        <is>
-          <t>Keep secrets out</t>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Start with contacts and meeting/pickup plans; medications, allergies and essential equipment; insurance and health information; locations of identity/legal documents; dependant or pet arrangements; and the emergency-kit / exit plan. That first pass is useful on its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="21" customHeight="1">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Keep private details safe</t>
         </is>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
-      <c r="B16" s="28" t="inlineStr">
-        <is>
-          <t>Do not put passwords, PINs, recovery codes or security answers here. Write where to find the information, not the secret itself.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="B18" s="25" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Do not enter passwords, PINs or recovery codes. In a location field, name the folder, safe place or person to ask, not the secret itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Ten-minute test</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="B19" s="26" t="inlineStr">
-        <is>
-          <t>Could someone you trust find your emergency contacts, medication information, insurance details, important-document locations and care arrangements without your phone or explanation?</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Could someone you trust find the emergency contacts, medication information, insurance details, document locations and care arrangements without your phone or help?</t>
+        </is>
+      </c>
+    </row>
     <row r="21" ht="36" customHeight="1">
-      <c r="B21" s="29" t="inlineStr">
-        <is>
-          <t>Anything hard to find is a useful place to start improving the checklist.</t>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>When something is hard to find, improve the instructions or access before making more copies.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B5:C5"/>
   </mergeCells>
@@ -830,650 +716,650 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="30" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="B1" s="30" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Item / information</t>
         </is>
       </c>
-      <c r="C1" s="30" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>What ready looks like</t>
         </is>
       </c>
-      <c r="D1" s="30" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Applies?</t>
         </is>
       </c>
-      <c r="E1" s="30" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Ready?</t>
         </is>
       </c>
-      <c r="F1" s="30" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Where to find it / who knows</t>
         </is>
       </c>
-      <c r="G1" s="30" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
       </c>
     </row>
     <row r="2" ht="58" customHeight="1">
-      <c r="A2" s="31" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Contacts &amp; coordination</t>
         </is>
       </c>
-      <c r="B2" s="32" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Primary household emergency contacts</t>
         </is>
       </c>
-      <c r="C2" s="31" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>Keep current names and phone numbers or another reliable way to reach them; anyone who may use the plan should know where it is.</t>
         </is>
       </c>
-      <c r="D2" s="33" t="inlineStr"/>
-      <c r="E2" s="33" t="inlineStr"/>
-      <c r="F2" s="31" t="inlineStr"/>
-      <c r="G2" s="34" t="inlineStr"/>
+      <c r="D2" s="14" t="inlineStr"/>
+      <c r="E2" s="14" t="inlineStr"/>
+      <c r="F2" s="12" t="inlineStr"/>
+      <c r="G2" s="15" t="inlineStr"/>
     </row>
     <row r="3" ht="58" customHeight="1">
-      <c r="A3" s="31" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Contacts &amp; coordination</t>
         </is>
       </c>
-      <c r="B3" s="32" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Out-of-area contact</t>
         </is>
       </c>
-      <c r="C3" s="31" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>Keep one current person outside your immediate area who household members can contact if local people are separated.</t>
         </is>
       </c>
-      <c r="D3" s="33" t="inlineStr"/>
-      <c r="E3" s="33" t="inlineStr"/>
-      <c r="F3" s="31" t="inlineStr"/>
-      <c r="G3" s="34" t="inlineStr"/>
+      <c r="D3" s="14" t="inlineStr"/>
+      <c r="E3" s="14" t="inlineStr"/>
+      <c r="F3" s="12" t="inlineStr"/>
+      <c r="G3" s="15" t="inlineStr"/>
     </row>
     <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="31" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Contacts &amp; coordination</t>
         </is>
       </c>
-      <c r="B4" s="32" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Meeting places</t>
         </is>
       </c>
-      <c r="C4" s="31" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Record the places household members should use if home is unavailable or people are separated.</t>
         </is>
       </c>
-      <c r="D4" s="33" t="inlineStr"/>
-      <c r="E4" s="33" t="inlineStr"/>
-      <c r="F4" s="31" t="inlineStr"/>
-      <c r="G4" s="34" t="inlineStr"/>
+      <c r="D4" s="14" t="inlineStr"/>
+      <c r="E4" s="14" t="inlineStr"/>
+      <c r="F4" s="12" t="inlineStr"/>
+      <c r="G4" s="15" t="inlineStr"/>
     </row>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="31" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Contacts &amp; coordination</t>
         </is>
       </c>
-      <c r="B5" s="32" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Trusted person who can find key information</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>Someone you trust should know the plan exists and where to start if you are unavailable.</t>
         </is>
       </c>
-      <c r="D5" s="33" t="inlineStr"/>
-      <c r="E5" s="33" t="inlineStr"/>
-      <c r="F5" s="31" t="inlineStr"/>
-      <c r="G5" s="34" t="inlineStr"/>
+      <c r="D5" s="14" t="inlineStr"/>
+      <c r="E5" s="14" t="inlineStr"/>
+      <c r="F5" s="12" t="inlineStr"/>
+      <c r="G5" s="15" t="inlineStr"/>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Contacts &amp; coordination</t>
         </is>
       </c>
-      <c r="B6" s="32" t="inlineStr">
-        <is>
-          <t>Local emergency / non-emergency information</t>
-        </is>
-      </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Useful local emergency numbers and information</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>Keep only the local numbers or official information sources that are genuinely useful where you live.</t>
         </is>
       </c>
-      <c r="D6" s="33" t="inlineStr"/>
-      <c r="E6" s="33" t="inlineStr"/>
-      <c r="F6" s="31" t="inlineStr"/>
-      <c r="G6" s="34" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr"/>
+      <c r="F6" s="12" t="inlineStr"/>
+      <c r="G6" s="15" t="inlineStr"/>
     </row>
     <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="31" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Health &amp; care</t>
         </is>
       </c>
-      <c r="B7" s="32" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Current medication list</t>
         </is>
       </c>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Keep a current, readable list accessible. Include the medication name, dosage/frequency and purpose when useful; this does not replace prescriptions or medical records.</t>
         </is>
       </c>
-      <c r="D7" s="33" t="inlineStr"/>
-      <c r="E7" s="33" t="inlineStr"/>
-      <c r="F7" s="31" t="inlineStr"/>
-      <c r="G7" s="34" t="inlineStr"/>
+      <c r="D7" s="14" t="inlineStr"/>
+      <c r="E7" s="14" t="inlineStr"/>
+      <c r="F7" s="12" t="inlineStr"/>
+      <c r="G7" s="15" t="inlineStr"/>
     </row>
     <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="31" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Health &amp; care</t>
         </is>
       </c>
-      <c r="B8" s="32" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Allergies and critical health information</t>
         </is>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Keep the minimum information another household member, trusted person or caregiver may need quickly, and update it when health circumstances change.</t>
         </is>
       </c>
-      <c r="D8" s="33" t="inlineStr"/>
-      <c r="E8" s="33" t="inlineStr"/>
-      <c r="F8" s="31" t="inlineStr"/>
-      <c r="G8" s="34" t="inlineStr"/>
+      <c r="D8" s="14" t="inlineStr"/>
+      <c r="E8" s="14" t="inlineStr"/>
+      <c r="F8" s="12" t="inlineStr"/>
+      <c r="G8" s="15" t="inlineStr"/>
     </row>
     <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Health &amp; care</t>
         </is>
       </c>
-      <c r="B9" s="32" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Medical devices, equipment or essential supplies</t>
         </is>
       </c>
-      <c r="C9" s="31" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Know what is needed, where it is, how it is used or moved, and any power or supply needs that matter during a disruption.</t>
         </is>
       </c>
-      <c r="D9" s="33" t="inlineStr"/>
-      <c r="E9" s="33" t="inlineStr"/>
-      <c r="F9" s="31" t="inlineStr"/>
-      <c r="G9" s="34" t="inlineStr"/>
+      <c r="D9" s="14" t="inlineStr"/>
+      <c r="E9" s="14" t="inlineStr"/>
+      <c r="F9" s="12" t="inlineStr"/>
+      <c r="G9" s="15" t="inlineStr"/>
     </row>
     <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Health &amp; care</t>
         </is>
       </c>
-      <c r="B10" s="32" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Doctor, clinic and pharmacy contacts</t>
         </is>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>Keep current phone numbers or other reliable contact details if these providers matter to the household.</t>
         </is>
       </c>
-      <c r="D10" s="33" t="inlineStr"/>
-      <c r="E10" s="33" t="inlineStr"/>
-      <c r="F10" s="31" t="inlineStr"/>
-      <c r="G10" s="34" t="inlineStr"/>
+      <c r="D10" s="14" t="inlineStr"/>
+      <c r="E10" s="14" t="inlineStr"/>
+      <c r="F10" s="12" t="inlineStr"/>
+      <c r="G10" s="15" t="inlineStr"/>
     </row>
     <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Health &amp; care</t>
         </is>
       </c>
-      <c r="B11" s="32" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Care, accessibility or support instructions</t>
         </is>
       </c>
-      <c r="C11" s="31" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>Write down the practical information someone would need to support a household member safely if normal help is disrupted.</t>
         </is>
       </c>
-      <c r="D11" s="33" t="inlineStr"/>
-      <c r="E11" s="33" t="inlineStr"/>
-      <c r="F11" s="31" t="inlineStr"/>
-      <c r="G11" s="34" t="inlineStr"/>
+      <c r="D11" s="14" t="inlineStr"/>
+      <c r="E11" s="14" t="inlineStr"/>
+      <c r="F11" s="12" t="inlineStr"/>
+      <c r="G11" s="15" t="inlineStr"/>
     </row>
     <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Health &amp; care</t>
         </is>
       </c>
-      <c r="B12" s="32" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Health card / coverage location</t>
         </is>
       </c>
-      <c r="C12" s="31" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>Know where the current card or official record is. Keep only the minimum useful reference details accessible.</t>
         </is>
       </c>
-      <c r="D12" s="33" t="inlineStr"/>
-      <c r="E12" s="33" t="inlineStr"/>
-      <c r="F12" s="31" t="inlineStr"/>
-      <c r="G12" s="34" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr"/>
+      <c r="E12" s="14" t="inlineStr"/>
+      <c r="F12" s="12" t="inlineStr"/>
+      <c r="G12" s="15" t="inlineStr"/>
     </row>
     <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Identity &amp; legal</t>
         </is>
       </c>
-      <c r="B13" s="32" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Passports and government-issued identification</t>
         </is>
       </c>
-      <c r="C13" s="31" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>Know where current originals are kept. Use a copy only when it is useful and appropriate; a copy does not replace the original.</t>
         </is>
       </c>
-      <c r="D13" s="33" t="inlineStr"/>
-      <c r="E13" s="33" t="inlineStr"/>
-      <c r="F13" s="31" t="inlineStr"/>
-      <c r="G13" s="34" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr"/>
+      <c r="F13" s="12" t="inlineStr"/>
+      <c r="G13" s="15" t="inlineStr"/>
     </row>
     <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Identity &amp; legal</t>
         </is>
       </c>
-      <c r="B14" s="32" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>Birth, citizenship or immigration documents</t>
         </is>
       </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>Know where the originals are kept. Do not carry them in a general emergency folder unless needed.</t>
-        </is>
-      </c>
-      <c r="D14" s="33" t="inlineStr"/>
-      <c r="E14" s="33" t="inlineStr"/>
-      <c r="F14" s="31" t="inlineStr"/>
-      <c r="G14" s="34" t="inlineStr"/>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Know the secure location of applicable originals; avoid carrying originals unnecessarily in a general emergency folder.</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr"/>
+      <c r="F14" s="12" t="inlineStr"/>
+      <c r="G14" s="15" t="inlineStr"/>
     </row>
     <row r="15" ht="58" customHeight="1">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Identity &amp; legal</t>
         </is>
       </c>
-      <c r="B15" s="32" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Will, power of attorney, personal directive or similar document</t>
         </is>
       </c>
-      <c r="C15" s="31" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>If applicable, someone you trust should know what exists and where the current signed or official document is kept. This checklist does not create legal authority.</t>
         </is>
       </c>
-      <c r="D15" s="33" t="inlineStr"/>
-      <c r="E15" s="33" t="inlineStr"/>
-      <c r="F15" s="31" t="inlineStr"/>
-      <c r="G15" s="34" t="inlineStr"/>
+      <c r="D15" s="14" t="inlineStr"/>
+      <c r="E15" s="14" t="inlineStr"/>
+      <c r="F15" s="12" t="inlineStr"/>
+      <c r="G15" s="15" t="inlineStr"/>
     </row>
     <row r="16" ht="58" customHeight="1">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Identity &amp; legal</t>
         </is>
       </c>
-      <c r="B16" s="32" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Custody, guardianship or consent documents</t>
         </is>
       </c>
-      <c r="C16" s="31" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>If applicable, know where the current document is kept and keep the practical information needed for emergency care or authorized pickup easy to find.</t>
         </is>
       </c>
-      <c r="D16" s="33" t="inlineStr"/>
-      <c r="E16" s="33" t="inlineStr"/>
-      <c r="F16" s="31" t="inlineStr"/>
-      <c r="G16" s="34" t="inlineStr"/>
+      <c r="D16" s="14" t="inlineStr"/>
+      <c r="E16" s="14" t="inlineStr"/>
+      <c r="F16" s="12" t="inlineStr"/>
+      <c r="G16" s="15" t="inlineStr"/>
     </row>
     <row r="17" ht="58" customHeight="1">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Insurance &amp; financial references</t>
         </is>
       </c>
-      <c r="B17" s="32" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Home / tenant / vehicle insurance</t>
         </is>
       </c>
-      <c r="C17" s="31" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>Keep the current insurer, policy reference and claims phone number easy to find; the full policy can stay in its normal secure location.</t>
         </is>
       </c>
-      <c r="D17" s="33" t="inlineStr"/>
-      <c r="E17" s="33" t="inlineStr"/>
-      <c r="F17" s="31" t="inlineStr"/>
-      <c r="G17" s="34" t="inlineStr"/>
+      <c r="D17" s="14" t="inlineStr"/>
+      <c r="E17" s="14" t="inlineStr"/>
+      <c r="F17" s="12" t="inlineStr"/>
+      <c r="G17" s="15" t="inlineStr"/>
     </row>
     <row r="18" ht="58" customHeight="1">
-      <c r="A18" s="31" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Insurance &amp; financial references</t>
         </is>
       </c>
-      <c r="B18" s="32" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Other relevant insurance</t>
         </is>
       </c>
-      <c r="C18" s="31" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>For life, health, travel, pet or other applicable coverage, keep enough information to identify the current provider and policy.</t>
         </is>
       </c>
-      <c r="D18" s="33" t="inlineStr"/>
-      <c r="E18" s="33" t="inlineStr"/>
-      <c r="F18" s="31" t="inlineStr"/>
-      <c r="G18" s="34" t="inlineStr"/>
+      <c r="D18" s="14" t="inlineStr"/>
+      <c r="E18" s="14" t="inlineStr"/>
+      <c r="F18" s="12" t="inlineStr"/>
+      <c r="G18" s="15" t="inlineStr"/>
     </row>
     <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Insurance &amp; financial references</t>
         </is>
       </c>
-      <c r="B19" s="32" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Banking and essential financial contacts</t>
         </is>
       </c>
-      <c r="C19" s="31" t="inlineStr">
-        <is>
-          <t>Note the institutions to contact and where the current records are kept. Do not record passwords, PINs or recovery codes.</t>
-        </is>
-      </c>
-      <c r="D19" s="33" t="inlineStr"/>
-      <c r="E19" s="33" t="inlineStr"/>
-      <c r="F19" s="31" t="inlineStr"/>
-      <c r="G19" s="34" t="inlineStr"/>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Know which institutions matter and where current records are kept. If you keep a reference accessible, use only what is actually needed; do not record passwords, PINs or recovery codes here.</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr"/>
+      <c r="E19" s="14" t="inlineStr"/>
+      <c r="F19" s="12" t="inlineStr"/>
+      <c r="G19" s="15" t="inlineStr"/>
     </row>
     <row r="20" ht="58" customHeight="1">
-      <c r="A20" s="31" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Children, dependants &amp; pets</t>
         </is>
       </c>
-      <c r="B20" s="32" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>School / daycare emergency and pickup arrangements</t>
         </is>
       </c>
-      <c r="C20" s="31" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>If applicable, keep current school/daycare contact information and the authorized pickup plan easy to find.</t>
         </is>
       </c>
-      <c r="D20" s="33" t="inlineStr"/>
-      <c r="E20" s="33" t="inlineStr"/>
-      <c r="F20" s="31" t="inlineStr"/>
-      <c r="G20" s="34" t="inlineStr"/>
+      <c r="D20" s="14" t="inlineStr"/>
+      <c r="E20" s="14" t="inlineStr"/>
+      <c r="F20" s="12" t="inlineStr"/>
+      <c r="G20" s="15" t="inlineStr"/>
     </row>
     <row r="21" ht="58" customHeight="1">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Children, dependants &amp; pets</t>
         </is>
       </c>
-      <c r="B21" s="32" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Dependant care instructions</t>
         </is>
       </c>
-      <c r="C21" s="31" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>Keep current practical care information for children, older relatives or other dependants someone may need to support.</t>
         </is>
       </c>
-      <c r="D21" s="33" t="inlineStr"/>
-      <c r="E21" s="33" t="inlineStr"/>
-      <c r="F21" s="31" t="inlineStr"/>
-      <c r="G21" s="34" t="inlineStr"/>
+      <c r="D21" s="14" t="inlineStr"/>
+      <c r="E21" s="14" t="inlineStr"/>
+      <c r="F21" s="12" t="inlineStr"/>
+      <c r="G21" s="15" t="inlineStr"/>
     </row>
     <row r="22" ht="58" customHeight="1">
-      <c r="A22" s="31" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>Children, dependants &amp; pets</t>
         </is>
       </c>
-      <c r="B22" s="32" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Support network for disability or special needs</t>
         </is>
       </c>
-      <c r="C22" s="31" t="inlineStr">
+      <c r="C22" s="12" t="inlineStr">
         <is>
           <t>If applicable, identify the people, equipment, supplies and practical instructions that matter when normal support is disrupted.</t>
         </is>
       </c>
-      <c r="D22" s="33" t="inlineStr"/>
-      <c r="E22" s="33" t="inlineStr"/>
-      <c r="F22" s="31" t="inlineStr"/>
-      <c r="G22" s="34" t="inlineStr"/>
+      <c r="D22" s="14" t="inlineStr"/>
+      <c r="E22" s="14" t="inlineStr"/>
+      <c r="F22" s="12" t="inlineStr"/>
+      <c r="G22" s="15" t="inlineStr"/>
     </row>
     <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Children, dependants &amp; pets</t>
         </is>
       </c>
-      <c r="B23" s="32" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Pet / service-animal identification and care information</t>
         </is>
       </c>
-      <c r="C23" s="31" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>Keep current identification, veterinarian details, medications, vaccination/licence references and other useful care information.</t>
         </is>
       </c>
-      <c r="D23" s="33" t="inlineStr"/>
-      <c r="E23" s="33" t="inlineStr"/>
-      <c r="F23" s="31" t="inlineStr"/>
-      <c r="G23" s="34" t="inlineStr"/>
+      <c r="D23" s="14" t="inlineStr"/>
+      <c r="E23" s="14" t="inlineStr"/>
+      <c r="F23" s="12" t="inlineStr"/>
+      <c r="G23" s="15" t="inlineStr"/>
     </row>
     <row r="24" ht="58" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Children, dependants &amp; pets</t>
         </is>
       </c>
-      <c r="B24" s="32" t="inlineStr">
-        <is>
-          <t>Where your pet or service animal can go</t>
-        </is>
-      </c>
-      <c r="C24" s="31" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Pet / service-animal evacuation destination</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>Know where the animal can go and what transport, carrier or accommodation arrangements are needed.</t>
         </is>
       </c>
-      <c r="D24" s="33" t="inlineStr"/>
-      <c r="E24" s="33" t="inlineStr"/>
-      <c r="F24" s="31" t="inlineStr"/>
-      <c r="G24" s="34" t="inlineStr"/>
+      <c r="D24" s="14" t="inlineStr"/>
+      <c r="E24" s="14" t="inlineStr"/>
+      <c r="F24" s="12" t="inlineStr"/>
+      <c r="G24" s="15" t="inlineStr"/>
     </row>
     <row r="25" ht="58" customHeight="1">
-      <c r="A25" s="31" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Home &amp; evacuation basics</t>
         </is>
       </c>
-      <c r="B25" s="32" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>Safe exits / evacuation route</t>
         </is>
       </c>
-      <c r="C25" s="31" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>Household members should know the relevant exits and how to leave the area; follow current local authority instructions during an actual emergency.</t>
         </is>
       </c>
-      <c r="D25" s="33" t="inlineStr"/>
-      <c r="E25" s="33" t="inlineStr"/>
-      <c r="F25" s="31" t="inlineStr"/>
-      <c r="G25" s="34" t="inlineStr"/>
+      <c r="D25" s="14" t="inlineStr"/>
+      <c r="E25" s="14" t="inlineStr"/>
+      <c r="F25" s="12" t="inlineStr"/>
+      <c r="G25" s="15" t="inlineStr"/>
     </row>
     <row r="26" ht="58" customHeight="1">
-      <c r="A26" s="31" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Home &amp; evacuation basics</t>
         </is>
       </c>
-      <c r="B26" s="32" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>Emergency kit / grab-and-go kit location</t>
         </is>
       </c>
-      <c r="C26" s="31" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>Everyone who may need the kit should know where it is kept.</t>
         </is>
       </c>
-      <c r="D26" s="33" t="inlineStr"/>
-      <c r="E26" s="33" t="inlineStr"/>
-      <c r="F26" s="31" t="inlineStr"/>
-      <c r="G26" s="34" t="inlineStr"/>
+      <c r="D26" s="14" t="inlineStr"/>
+      <c r="E26" s="14" t="inlineStr"/>
+      <c r="F26" s="12" t="inlineStr"/>
+      <c r="G26" s="15" t="inlineStr"/>
     </row>
     <row r="27" ht="58" customHeight="1">
-      <c r="A27" s="31" t="inlineStr">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Home &amp; evacuation basics</t>
         </is>
       </c>
-      <c r="B27" s="32" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Fire extinguisher and key safety equipment locations</t>
         </is>
       </c>
-      <c r="C27" s="31" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>Know where the equipment is. This checklist does not replace training, product instructions or emergency-service guidance.</t>
         </is>
       </c>
-      <c r="D27" s="33" t="inlineStr"/>
-      <c r="E27" s="33" t="inlineStr"/>
-      <c r="F27" s="31" t="inlineStr"/>
-      <c r="G27" s="34" t="inlineStr"/>
+      <c r="D27" s="14" t="inlineStr"/>
+      <c r="E27" s="14" t="inlineStr"/>
+      <c r="F27" s="12" t="inlineStr"/>
+      <c r="G27" s="15" t="inlineStr"/>
     </row>
     <row r="28" ht="58" customHeight="1">
-      <c r="A28" s="31" t="inlineStr">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>Home &amp; evacuation basics</t>
         </is>
       </c>
-      <c r="B28" s="32" t="inlineStr">
-        <is>
-          <t>Water, electricity, gas and heating controls</t>
-        </is>
-      </c>
-      <c r="C28" s="31" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Water, electrical, gas / heating and other utility controls</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>Know where the controls are and who to contact. Do not improvise shutoff procedures during an emergency.</t>
         </is>
       </c>
-      <c r="D28" s="33" t="inlineStr"/>
-      <c r="E28" s="33" t="inlineStr"/>
-      <c r="F28" s="31" t="inlineStr"/>
-      <c r="G28" s="34" t="inlineStr"/>
+      <c r="D28" s="14" t="inlineStr"/>
+      <c r="E28" s="14" t="inlineStr"/>
+      <c r="F28" s="12" t="inlineStr"/>
+      <c r="G28" s="15" t="inlineStr"/>
     </row>
     <row r="29" ht="58" customHeight="1">
-      <c r="A29" s="31" t="inlineStr">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>Home &amp; evacuation basics</t>
         </is>
       </c>
-      <c r="B29" s="32" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Landlord, building management or property contact</t>
         </is>
       </c>
-      <c r="C29" s="31" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>If applicable, keep a current phone number or other reliable way to reach the person or service responsible.</t>
         </is>
       </c>
-      <c r="D29" s="33" t="inlineStr"/>
-      <c r="E29" s="33" t="inlineStr"/>
-      <c r="F29" s="31" t="inlineStr"/>
-      <c r="G29" s="34" t="inlineStr"/>
+      <c r="D29" s="14" t="inlineStr"/>
+      <c r="E29" s="14" t="inlineStr"/>
+      <c r="F29" s="12" t="inlineStr"/>
+      <c r="G29" s="15" t="inlineStr"/>
     </row>
     <row r="30" ht="58" customHeight="1">
-      <c r="A30" s="31" t="inlineStr">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>Home &amp; evacuation basics</t>
         </is>
       </c>
-      <c r="B30" s="32" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Local hazards and official alerts</t>
         </is>
       </c>
-      <c r="C30" s="31" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>Know which hazards are realistic where you live and which official sources provide warnings or instructions.</t>
         </is>
       </c>
-      <c r="D30" s="33" t="inlineStr"/>
-      <c r="E30" s="33" t="inlineStr"/>
-      <c r="F30" s="31" t="inlineStr"/>
-      <c r="G30" s="34" t="inlineStr"/>
+      <c r="D30" s="14" t="inlineStr"/>
+      <c r="E30" s="14" t="inlineStr"/>
+      <c r="F30" s="12" t="inlineStr"/>
+      <c r="G30" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G30"/>
@@ -1504,29 +1390,29 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="35" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Trigger</t>
         </is>
       </c>
-      <c r="B1" s="35" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Review when…</t>
         </is>
       </c>
-      <c r="C1" s="35" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>Checked</t>
         </is>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="36" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>Contact changes</t>
         </is>
       </c>
-      <c r="B2" s="26" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Phone number, address, trusted contact, provider or emergency contact changes.</t>
         </is>
@@ -1534,12 +1420,12 @@
       <c r="C2" s="18" t="inlineStr"/>
     </row>
     <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="36" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Health changes</t>
         </is>
       </c>
-      <c r="B3" s="26" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Medication, allergy, condition, medical-device, care or accessibility needs change.</t>
         </is>
@@ -1547,12 +1433,12 @@
       <c r="C3" s="18" t="inlineStr"/>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="36" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Household changes</t>
         </is>
       </c>
-      <c r="B4" s="26" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Someone joins or leaves the household; a dependant or caregiver arrangement changes.</t>
         </is>
@@ -1560,12 +1446,12 @@
       <c r="C4" s="18" t="inlineStr"/>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="36" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>School / care changes</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>School, daycare, pickup authorization, custody or support arrangements change.</t>
         </is>
@@ -1573,12 +1459,12 @@
       <c r="C5" s="18" t="inlineStr"/>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Insurance changes</t>
         </is>
       </c>
-      <c r="B6" s="26" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>A policy renews, provider changes, coverage changes or claim information changes.</t>
         </is>
@@ -1586,12 +1472,12 @@
       <c r="C6" s="18" t="inlineStr"/>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="36" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Identity / legal changes</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Passport or ID renews; a legal document is created, amended, revoked or moved.</t>
         </is>
@@ -1599,12 +1485,12 @@
       <c r="C7" s="18" t="inlineStr"/>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Pet changes</t>
         </is>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Pet medication, veterinarian, licence, microchip, boarding or evacuation arrangements change.</t>
         </is>
@@ -1612,12 +1498,12 @@
       <c r="C8" s="18" t="inlineStr"/>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Home / move changes</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Address, building, utility, landlord, emergency-kit location or evacuation route changes.</t>
         </is>
@@ -1625,12 +1511,12 @@
       <c r="C9" s="18" t="inlineStr"/>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="36" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>After an emergency or drill</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Something was hard to find, unclear, out of date or inaccessible when tested.</t>
         </is>
@@ -1638,12 +1524,12 @@
       <c r="C10" s="18" t="inlineStr"/>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="36" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Periodic refresh</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Even if nothing obvious changed, do a quick review once or twice a year to catch expiry, stale contacts and quiet changes.</t>
         </is>
@@ -1674,122 +1560,122 @@
   </cols>
   <sheetData>
     <row r="1" ht="52" customHeight="1">
-      <c r="A1" s="29" t="inlineStr">
-        <is>
-          <t>What this helps with</t>
-        </is>
-      </c>
-      <c r="B1" s="26" t="inlineStr">
-        <is>
-          <t>Find the household contacts and information you may need in the first minutes and hours of an emergency.</t>
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>A practical checklist for finding essential household information in the first minutes and hours of an emergency.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="52" customHeight="1">
-      <c r="A2" s="29" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Not included</t>
         </is>
       </c>
-      <c r="B2" s="26" t="inlineStr">
-        <is>
-          <t>Use the Household Information Plan for ongoing bills, claims, unfinished tasks and responsibilities over the following days and weeks.</t>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>For ongoing bills, claims, accounts and unfinished tasks, use the separate household information plan.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="29" t="inlineStr">
-        <is>
-          <t>Use what applies</t>
-        </is>
-      </c>
-      <c r="B3" s="26" t="inlineStr">
-        <is>
-          <t>Skip anything your household does not need.</t>
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>What applies</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Skip anything that does not apply to your household.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Originals and copies</t>
         </is>
       </c>
-      <c r="B4" s="26" t="inlineStr">
-        <is>
-          <t>A copy or note about a document does not replace the original or give someone legal permission to act.</t>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>A copy, summary or location note does not replace an original document or give someone legal permission to act.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr">
-        <is>
-          <t>Do not record passwords, PINs, recovery codes or security answers. Keep sensitive originals in a secure place.</t>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Do not record passwords, PINs, recovery codes, full credentials or unnecessary account secrets. Avoid concentrating every sensitive original in one portable place.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="29" t="inlineStr">
-        <is>
-          <t>Government of Canada: household plan</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Government of Canada: household plan</t>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Government of Canada : household plan</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>Open the official guidance</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="29" t="inlineStr">
-        <is>
-          <t>Government of Canada: emergency kit</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>Government of Canada: emergency kit</t>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Government of Canada : emergency kit</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Open the official guidance</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
-        <is>
-          <t>Government of Canada: disabilities</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>Government of Canada: disabilities</t>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Government of Canada : disabilities</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>Open the official guidance</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="29" t="inlineStr">
-        <is>
-          <t>Government of Canada: pets and service animals</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>Government of Canada: pets and service animals</t>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Government of Canada : pets / service animals</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>Open the official guidance</t>
         </is>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="29" t="inlineStr">
-        <is>
-          <t>Version and reuse</t>
-        </is>
-      </c>
-      <c r="B10" s="26" t="inlineStr">
-        <is>
-          <t>Version 0.1.1, reviewed 17 September 2026. This maintenance edition retains the existing CC BY 4.0 licence for Eterna-authored checklist content. See LICENSE-NOTICE.md.</t>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Maintenance candidate 0.1.1. Original resource content retains its existing CC BY 4.0 terms. See LICENSE-NOTICE.md. Public release remains subject to review.</t>
         </is>
       </c>
     </row>

</xml_diff>